<commit_message>
deploying onto the server
</commit_message>
<xml_diff>
--- a/nse_option_chain.xlsx
+++ b/nse_option_chain.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>7.58</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.53</t>
+          <t>4.59</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>7.46</t>
+          <t>7.37</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>14.32</t>
+          <t>14.35</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">

</xml_diff>